<commit_message>
Added more files to digital files
</commit_message>
<xml_diff>
--- a/data/AfSdemo_DigitalResources_20260813ale.xlsx
+++ b/data/AfSdemo_DigitalResources_20260813ale.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="4"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="3"/>
   </bookViews>
   <sheets>
     <sheet name="name" sheetId="1" state="visible" r:id="rId3"/>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="453" uniqueCount="180">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="522" uniqueCount="248">
   <si>
     <t xml:space="preserve">resourceinstance_id</t>
   </si>
@@ -197,211 +197,415 @@
     <t xml:space="preserve">file</t>
   </si>
   <si>
+    <t xml:space="preserve">file_uuid</t>
+  </si>
+  <si>
     <t xml:space="preserve">VioBiolk_flat.rpl</t>
   </si>
   <si>
+    <t xml:space="preserve"> 33b8b921-034d-4422-8841-d30176ad995e</t>
+  </si>
+  <si>
     <t xml:space="preserve">VioBiolk_flat.bcf</t>
   </si>
   <si>
+    <t xml:space="preserve"> c0c0dc86-4f10-4cc1-af1b-adde2b0782fc</t>
+  </si>
+  <si>
     <t xml:space="preserve">VioBiolk_flat.raw</t>
   </si>
   <si>
+    <t xml:space="preserve"> cea6aefd-6001-4915-93e3-910a71164a0e</t>
+  </si>
+  <si>
     <t xml:space="preserve">Biolk_XRF__001.spx</t>
   </si>
   <si>
+    <t xml:space="preserve"> ed2d2e43-74b2-409b-8c95-4a770ad38bc4</t>
+  </si>
+  <si>
     <t xml:space="preserve">Biolk_XRF__001minus008.spx</t>
   </si>
   <si>
+    <t xml:space="preserve"> b7b78332-37b6-402c-a76d-e843ad5e2880</t>
+  </si>
+  <si>
     <t xml:space="preserve">Biolk_XRF__001.txt</t>
   </si>
   <si>
+    <t xml:space="preserve"> 37d8bc63-dd9c-4bf6-90cd-41e947532537</t>
+  </si>
+  <si>
     <t xml:space="preserve">Biolk_XRF__001minus008.txt</t>
   </si>
   <si>
+    <t xml:space="preserve"> 49a392bf-096a-4469-bde4-b72320b87e03</t>
+  </si>
+  <si>
     <t xml:space="preserve">Biolk_XRF__005minus008.txt</t>
   </si>
   <si>
+    <t xml:space="preserve"> 198efb7a-bee3-4c0b-aa03-4c124e04519c</t>
+  </si>
+  <si>
     <t xml:space="preserve">Biolk_XRF__005minus008.spx</t>
   </si>
   <si>
+    <t xml:space="preserve"> c0b934e7-196b-4f9a-b10f-311e2469ca7f</t>
+  </si>
+  <si>
     <t xml:space="preserve">Biolk_XRF__005.spx</t>
   </si>
   <si>
+    <t xml:space="preserve"> 20ab2573-85cb-4042-922a-bcb1511ba625</t>
+  </si>
+  <si>
     <t xml:space="preserve">Biolk_XRF__005.txt</t>
   </si>
   <si>
+    <t xml:space="preserve"> a1d5ce40-7cb4-452c-afa6-4796cd795302</t>
+  </si>
+  <si>
     <t xml:space="preserve">Biolk_XRF__006.spx</t>
   </si>
   <si>
+    <t xml:space="preserve"> b2e5bad4-df49-4adc-83d5-150a474b9ef4</t>
+  </si>
+  <si>
     <t xml:space="preserve">Biolk_XRF__006minus008.spx</t>
   </si>
   <si>
+    <t xml:space="preserve"> 8170ccfd-d00c-4d69-9a39-29d7ce5e3057</t>
+  </si>
+  <si>
     <t xml:space="preserve">Biolk_XRF__006minus008.txt</t>
   </si>
   <si>
+    <t xml:space="preserve"> 880c0d00-d727-4859-a61d-9524335cc12c</t>
+  </si>
+  <si>
     <t xml:space="preserve">Biolk_XRF__006.txt</t>
   </si>
   <si>
+    <t xml:space="preserve"> 22dfd757-4142-49a8-ba15-383370bbb85e</t>
+  </si>
+  <si>
     <t xml:space="preserve">Biolk_XRF__004.txt</t>
   </si>
   <si>
+    <t xml:space="preserve"> b6666138-7306-4fe0-b0f5-aeed7e3c75e4</t>
+  </si>
+  <si>
     <t xml:space="preserve">Biolk_XRF__004minus008.spx</t>
   </si>
   <si>
+    <t xml:space="preserve"> 39374ef6-e1b1-4a58-b277-fac9a4919ffb</t>
+  </si>
+  <si>
     <t xml:space="preserve">Biolk_XRF__004.spx</t>
   </si>
   <si>
+    <t xml:space="preserve"> 725da319-238c-4f66-b93e-3809ef13c4a5</t>
+  </si>
+  <si>
     <t xml:space="preserve">Biolk_XRF__004minus008.txt</t>
   </si>
   <si>
+    <t xml:space="preserve"> 3b9cbc5c-01b5-4a59-a0dc-f0dfdcc5981b</t>
+  </si>
+  <si>
     <t xml:space="preserve">Biolk_XRF__008.spx</t>
   </si>
   <si>
+    <t xml:space="preserve"> f5506aac-a6ef-4fd5-a2dd-cba70afbe61e</t>
+  </si>
+  <si>
     <t xml:space="preserve">Biolk_XRF__008.txt</t>
   </si>
   <si>
+    <t xml:space="preserve"> 75dba810-82d0-4349-b9f2-c0073c974852</t>
+  </si>
+  <si>
     <t xml:space="preserve">Biolk_XRF__002minus008.spx</t>
   </si>
   <si>
+    <t xml:space="preserve"> 0bde8e88-72e3-4e98-a0c6-43a08903ec05</t>
+  </si>
+  <si>
     <t xml:space="preserve">Biolk_XRF__002.spx</t>
   </si>
   <si>
+    <t xml:space="preserve"> 7666c8ce-da9f-40d7-a101-937f85a50b0d</t>
+  </si>
+  <si>
     <t xml:space="preserve">Biolk_XRF__002.txt</t>
   </si>
   <si>
+    <t xml:space="preserve"> a88f5b03-4ae4-443d-ae45-2269e268a738</t>
+  </si>
+  <si>
     <t xml:space="preserve">Biolk_XRF__002minus008.txt</t>
   </si>
   <si>
+    <t xml:space="preserve"> 2f0d3d0b-8961-469c-a2c4-c2d89aac7035</t>
+  </si>
+  <si>
     <t xml:space="preserve">Biolk_XRF__003.spx</t>
   </si>
   <si>
+    <t xml:space="preserve"> e344d5b1-00da-4953-9145-ecea3d92f679</t>
+  </si>
+  <si>
     <t xml:space="preserve">Biolk_XRF__003.txt</t>
   </si>
   <si>
+    <t xml:space="preserve"> 5b9d5bc8-87f4-43d5-be8d-492720d16fd9</t>
+  </si>
+  <si>
     <t xml:space="preserve">Biolk_XRF__003minus008.spx</t>
   </si>
   <si>
+    <t xml:space="preserve"> c08cf678-6780-4bd2-a861-2fc1e4416574</t>
+  </si>
+  <si>
     <t xml:space="preserve">Biolk_XRF__003minus008.txt</t>
   </si>
   <si>
+    <t xml:space="preserve"> beaedb2b-c3f8-4a3e-8e12-37e223b3ffa9</t>
+  </si>
+  <si>
     <t xml:space="preserve">Biolk_XRF__007minus008.spx</t>
   </si>
   <si>
+    <t xml:space="preserve"> 7c65403f-c53d-44a9-b5ff-fb4ab4c65dd6</t>
+  </si>
+  <si>
     <t xml:space="preserve">Biolk_XRF__007.spx</t>
   </si>
   <si>
+    <t xml:space="preserve"> a4c29519-189e-464c-bf94-6ea5a33bb7a4</t>
+  </si>
+  <si>
     <t xml:space="preserve">Biolk_XRF__007minus008.txt</t>
   </si>
   <si>
+    <t xml:space="preserve"> 350bd7a3-f375-45db-b9f5-6ac9502796d1</t>
+  </si>
+  <si>
     <t xml:space="preserve">Biolk_XRF__007.txt</t>
   </si>
   <si>
+    <t xml:space="preserve"> 4dc73d16-5089-40d2-9936-e94bf4e6e32e</t>
+  </si>
+  <si>
     <t xml:space="preserve">TSR_FORS_biolk_00010.asd.sco.abs.dx</t>
   </si>
   <si>
+    <t xml:space="preserve"> ad209f79-c87c-4e4a-ba1a-048e5ad1e882</t>
+  </si>
+  <si>
     <t xml:space="preserve">TSR_FORS_biolk_00008.asd.sco.abs.dx</t>
   </si>
   <si>
+    <t xml:space="preserve"> fe5b89b6-234b-45a1-bf42-6d184449fa8a</t>
+  </si>
+  <si>
     <t xml:space="preserve">TSR_FORS_biolk_00003.asd.sco.abs.dx</t>
   </si>
   <si>
+    <t xml:space="preserve"> b457ba6f-98ea-488f-90d9-69263c5f16fb</t>
+  </si>
+  <si>
     <t xml:space="preserve">TSR_FORS_biolk_00007.asd.sco.abs.dx</t>
   </si>
   <si>
+    <t xml:space="preserve"> f229c70f-a3d2-4ea0-b398-060102faa3e8</t>
+  </si>
+  <si>
     <t xml:space="preserve">TSR_FORS_biolk_00009.asd.sco.abs.dx</t>
   </si>
   <si>
+    <t xml:space="preserve"> 52bbd3cc-06ce-45e0-85b7-509a0e9392de</t>
+  </si>
+  <si>
     <t xml:space="preserve">biolk_sC_100x_spot6.wxd</t>
   </si>
   <si>
+    <t xml:space="preserve"> a75ce363-5457-4e6f-9e81-98df0fe7f92b</t>
+  </si>
+  <si>
     <t xml:space="preserve">biolk_sC_100x_spot6.dx</t>
   </si>
   <si>
+    <t xml:space="preserve"> 5a36969a-3181-40c8-9cdb-0ba137bf08e6</t>
+  </si>
+  <si>
     <t xml:space="preserve">biolk_sC_100x_spot6.txt</t>
   </si>
   <si>
+    <t xml:space="preserve"> d916fea3-41f1-4029-a86f-0db99b993f4f</t>
+  </si>
+  <si>
     <t xml:space="preserve">biolk_sA2_20x_spot1.dx</t>
   </si>
   <si>
+    <t xml:space="preserve"> 6dbf2393-3721-4c89-9136-03ff7d035e0e</t>
+  </si>
+  <si>
     <t xml:space="preserve">biolk_sA2_50x_spot1.dx</t>
   </si>
   <si>
+    <t xml:space="preserve"> 65ababbc-d014-40a6-85ab-e31c227cdf70</t>
+  </si>
+  <si>
     <t xml:space="preserve">biolk_sA2_20x_spot1.wxd</t>
   </si>
   <si>
+    <t xml:space="preserve"> 37f6ac4e-c3bf-45ca-a170-746f156a9cdd</t>
+  </si>
+  <si>
     <t xml:space="preserve">biolk_sA2_20x_spot1.txt</t>
   </si>
   <si>
+    <t xml:space="preserve"> 81b996b9-b7d3-44e7-acc7-17182b5e1d2d</t>
+  </si>
+  <si>
     <t xml:space="preserve">biolk_sA2_50x_spot1.txt</t>
   </si>
   <si>
+    <t xml:space="preserve"> 8859f761-5c51-4d29-85b1-8064c9cdc563</t>
+  </si>
+  <si>
     <t xml:space="preserve">biolk_sA2_50x_spot1.wxd</t>
   </si>
   <si>
+    <t xml:space="preserve"> 3f04955c-82fb-4946-a972-e4b735db4c43</t>
+  </si>
+  <si>
     <t xml:space="preserve">biolk_sC_100x_spot5.txt</t>
   </si>
   <si>
+    <t xml:space="preserve"> 0d518d89-35e2-4319-aa0f-4d97c0fc0782</t>
+  </si>
+  <si>
     <t xml:space="preserve">biolk_sC_100x_spot5.dx</t>
   </si>
   <si>
+    <t xml:space="preserve"> d58d53df-c0ef-40a0-b60d-ef21361591c9</t>
+  </si>
+  <si>
     <t xml:space="preserve">biolk_sC_100x_spot5.wxd</t>
   </si>
   <si>
+    <t xml:space="preserve"> c24ca4d2-bcb2-4c40-a20c-642be1981fd5</t>
+  </si>
+  <si>
     <t xml:space="preserve">biolk_sA2_50x_spot2.dx</t>
   </si>
   <si>
+    <t xml:space="preserve"> 4fd97f19-c884-44d5-a63c-497ec66c79e8</t>
+  </si>
+  <si>
     <t xml:space="preserve">biolk_sA2_50x_spot2.txt</t>
   </si>
   <si>
+    <t xml:space="preserve"> b88a68aa-337a-4467-8470-f4d885064a61</t>
+  </si>
+  <si>
     <t xml:space="preserve">biolk_sA2_50x_spot2.wxd</t>
   </si>
   <si>
+    <t xml:space="preserve"> 133e2107-5e64-47ab-a588-48955ef1d427</t>
+  </si>
+  <si>
     <t xml:space="preserve">biolk_sA2_50x_spot3.dx</t>
   </si>
   <si>
+    <t xml:space="preserve"> b763a9ae-b23f-49d4-9da8-e1d3fca72f2d</t>
+  </si>
+  <si>
     <t xml:space="preserve">biolk_sA2_50x_spot3.txt</t>
   </si>
   <si>
+    <t xml:space="preserve"> dde74c8a-5357-4d8f-b6cd-d81208ed05ea</t>
+  </si>
+  <si>
     <t xml:space="preserve">biolk_sA2_50x_spot3.wxd</t>
   </si>
   <si>
+    <t xml:space="preserve"> edaecc1d-97ce-490d-95d3-0b3a4deea1d2</t>
+  </si>
+  <si>
     <t xml:space="preserve">biolk_sC_100x_spot4.dx</t>
   </si>
   <si>
+    <t xml:space="preserve"> c34a0b2b-3cd4-4c85-aa4f-1819ab2f71a6</t>
+  </si>
+  <si>
     <t xml:space="preserve">biolk_sC_100x_spot4.wxd</t>
   </si>
   <si>
+    <t xml:space="preserve"> 687e536f-9ea8-4b9f-9fd9-e8f9ec8ea35f</t>
+  </si>
+  <si>
     <t xml:space="preserve">biolk_sC_100x_spot4.txt</t>
   </si>
   <si>
+    <t xml:space="preserve"> 3f847aa1-441f-4063-ace6-947657c22b1d</t>
+  </si>
+  <si>
     <t xml:space="preserve">biolk_sC_100x_spot1.dx</t>
   </si>
   <si>
+    <t xml:space="preserve"> 6c4808b3-edab-44b5-96eb-f7512006153a</t>
+  </si>
+  <si>
     <t xml:space="preserve">biolk_sC_100x_spot1.txt</t>
   </si>
   <si>
+    <t xml:space="preserve"> 593a1ffe-68ae-48d5-8a42-341a60ecfe3c</t>
+  </si>
+  <si>
     <t xml:space="preserve">biolk_sC_100x_spot1.wxd</t>
   </si>
   <si>
+    <t xml:space="preserve"> 009fbff5-890d-4a7f-acd1-aa2764d5cf2f</t>
+  </si>
+  <si>
     <t xml:space="preserve">biolk_sC_100x_spot3.txt</t>
   </si>
   <si>
+    <t xml:space="preserve"> e091917a-3465-4de1-bffb-ef4b295a1f85</t>
+  </si>
+  <si>
     <t xml:space="preserve">biolk_sC_100x_spot3.wxd</t>
   </si>
   <si>
+    <t xml:space="preserve"> 62c68a62-4d3f-45fc-99eb-c69ff6ba31d1</t>
+  </si>
+  <si>
     <t xml:space="preserve">biolk_sC_100x_spot3.dx</t>
   </si>
   <si>
+    <t xml:space="preserve"> aeb2f3e0-72fe-486c-8b87-be52dc1135d9</t>
+  </si>
+  <si>
     <t xml:space="preserve">biolk_sC_100x_spot2.dx</t>
   </si>
   <si>
+    <t xml:space="preserve"> 69ca77fc-38e2-40be-9318-7079116d090f</t>
+  </si>
+  <si>
     <t xml:space="preserve">biolk_sC_100x_spot2.wxd</t>
   </si>
   <si>
+    <t xml:space="preserve"> a2be6af6-c9ad-40f0-b8ac-9569a7784fad</t>
+  </si>
+  <si>
     <t xml:space="preserve">biolk_sC_100x_spot2.txt</t>
   </si>
   <si>
-    <t xml:space="preserve">file_uuid</t>
+    <t xml:space="preserve"> e5a969d3-bdc5-450b-a050-675c66ff1dda</t>
   </si>
   <si>
     <t xml:space="preserve">file_statement_type</t>
@@ -640,12 +844,16 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -844,199 +1052,199 @@
   <dimension ref="A1:B24"/>
   <sheetFormatPr defaultColWidth="8.83203125" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="44.33"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="88"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="44.33"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="88"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="0" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="0" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="0" t="s">
+      <c r="A2" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="0" t="s">
+      <c r="B2" s="1" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="0" t="s">
+      <c r="A3" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B3" s="0" t="s">
+      <c r="B3" s="1" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="0" t="s">
+      <c r="A4" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="B4" s="0" t="s">
+      <c r="B4" s="1" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="0" t="s">
+      <c r="A5" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="B5" s="0" t="s">
+      <c r="B5" s="1" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="0" t="s">
+      <c r="A6" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="B6" s="0" t="s">
+      <c r="B6" s="1" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="0" t="s">
+      <c r="A7" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="B7" s="0" t="s">
+      <c r="B7" s="1" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="0" t="s">
+      <c r="A8" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="B8" s="0" t="s">
+      <c r="B8" s="1" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="0" t="s">
+      <c r="A9" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="B9" s="0" t="s">
+      <c r="B9" s="1" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="0" t="s">
+      <c r="A10" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="B10" s="0" t="s">
+      <c r="B10" s="1" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="0" t="s">
+      <c r="A11" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="B11" s="0" t="s">
+      <c r="B11" s="1" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="0" t="s">
+      <c r="A12" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="B12" s="0" t="s">
+      <c r="B12" s="1" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="0" t="s">
+      <c r="A13" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="B13" s="0" t="s">
+      <c r="B13" s="1" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="0" t="s">
+      <c r="A14" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="B14" s="0" t="s">
+      <c r="B14" s="1" t="s">
         <v>27</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="0" t="s">
+      <c r="A15" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="B15" s="0" t="s">
+      <c r="B15" s="1" t="s">
         <v>29</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="0" t="s">
+      <c r="A16" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="B16" s="0" t="s">
+      <c r="B16" s="1" t="s">
         <v>31</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="0" t="s">
+      <c r="A17" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="B17" s="0" t="s">
+      <c r="B17" s="1" t="s">
         <v>33</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="0" t="s">
+      <c r="A18" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="B18" s="0" t="s">
+      <c r="B18" s="1" t="s">
         <v>35</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="0" t="s">
+      <c r="A19" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="B19" s="0" t="s">
+      <c r="B19" s="1" t="s">
         <v>37</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="0" t="s">
+      <c r="A20" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="B20" s="0" t="s">
+      <c r="B20" s="1" t="s">
         <v>39</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="0" t="s">
+      <c r="A21" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="B21" s="0" t="s">
+      <c r="B21" s="1" t="s">
         <v>41</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="0" t="s">
+      <c r="A22" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="B22" s="0" t="s">
+      <c r="B22" s="1" t="s">
         <v>43</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="0" t="s">
+      <c r="A23" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="B23" s="0" t="s">
+      <c r="B23" s="1" t="s">
         <v>45</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="0" t="s">
+      <c r="A24" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="B24" s="0" t="s">
+      <c r="B24" s="1" t="s">
         <v>47</v>
       </c>
     </row>
@@ -1059,191 +1267,191 @@
   <dimension ref="A1:B23"/>
   <sheetFormatPr defaultColWidth="8.83203125" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="42.34"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="34.51"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="42.34"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="34.51"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="0" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="0" t="s">
+      <c r="B1" s="1" t="s">
         <v>48</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="0" t="s">
+      <c r="A2" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B2" s="0" t="s">
+      <c r="B2" s="1" t="s">
         <v>49</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="0" t="s">
+      <c r="A3" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="B3" s="0" t="s">
+      <c r="B3" s="1" t="s">
         <v>49</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="0" t="s">
+      <c r="A4" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="B4" s="0" t="s">
+      <c r="B4" s="1" t="s">
         <v>49</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="0" t="s">
+      <c r="A5" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="B5" s="0" t="s">
+      <c r="B5" s="1" t="s">
         <v>49</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="0" t="s">
+      <c r="A6" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="B6" s="0" t="s">
+      <c r="B6" s="1" t="s">
         <v>49</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="0" t="s">
+      <c r="A7" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="B7" s="0" t="s">
+      <c r="B7" s="1" t="s">
         <v>49</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="0" t="s">
+      <c r="A8" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="B8" s="0" t="s">
+      <c r="B8" s="1" t="s">
         <v>49</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="0" t="s">
+      <c r="A9" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="B9" s="0" t="s">
+      <c r="B9" s="1" t="s">
         <v>49</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="0" t="s">
+      <c r="A10" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="B10" s="0" t="s">
+      <c r="B10" s="1" t="s">
         <v>49</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="0" t="s">
+      <c r="A11" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="B11" s="0" t="s">
+      <c r="B11" s="1" t="s">
         <v>49</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="0" t="s">
+      <c r="A12" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="B12" s="0" t="s">
+      <c r="B12" s="1" t="s">
         <v>49</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="0" t="s">
+      <c r="A13" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="B13" s="0" t="s">
+      <c r="B13" s="1" t="s">
         <v>49</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="0" t="s">
+      <c r="A14" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="B14" s="0" t="s">
+      <c r="B14" s="1" t="s">
         <v>49</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="0" t="s">
+      <c r="A15" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="B15" s="0" t="s">
+      <c r="B15" s="1" t="s">
         <v>49</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="0" t="s">
+      <c r="A16" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="B16" s="0" t="s">
+      <c r="B16" s="1" t="s">
         <v>49</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="0" t="s">
+      <c r="A17" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="B17" s="0" t="s">
+      <c r="B17" s="1" t="s">
         <v>49</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="0" t="s">
+      <c r="A18" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="B18" s="0" t="s">
+      <c r="B18" s="1" t="s">
         <v>49</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="0" t="s">
+      <c r="A19" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="B19" s="0" t="s">
+      <c r="B19" s="1" t="s">
         <v>49</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="0" t="s">
+      <c r="A20" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="B20" s="0" t="s">
+      <c r="B20" s="1" t="s">
         <v>49</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="0" t="s">
+      <c r="A21" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="B21" s="0" t="s">
+      <c r="B21" s="1" t="s">
         <v>49</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="0" t="s">
+      <c r="A22" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="B22" s="0" t="s">
+      <c r="B22" s="1" t="s">
         <v>49</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="0" t="s">
+      <c r="A23" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="B23" s="0" t="s">
+      <c r="B23" s="1" t="s">
         <v>49</v>
       </c>
     </row>
@@ -1266,191 +1474,191 @@
   <dimension ref="A1:B23"/>
   <sheetFormatPr defaultColWidth="10.453125" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="43.33"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="36.5"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="43.33"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="36.5"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="0" t="s">
+      <c r="A1" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="B1" s="0" t="s">
+      <c r="B1" s="1" t="s">
         <v>51</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="0" t="s">
+      <c r="A2" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B2" s="0" t="s">
+      <c r="B2" s="1" t="s">
         <v>52</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="0" t="s">
+      <c r="A3" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="B3" s="0" t="s">
+      <c r="B3" s="1" t="s">
         <v>52</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="0" t="s">
+      <c r="A4" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="B4" s="0" t="s">
+      <c r="B4" s="1" t="s">
         <v>52</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="0" t="s">
+      <c r="A5" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="B5" s="0" t="s">
+      <c r="B5" s="1" t="s">
         <v>52</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="0" t="s">
+      <c r="A6" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="B6" s="0" t="s">
+      <c r="B6" s="1" t="s">
         <v>52</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="0" t="s">
+      <c r="A7" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="B7" s="0" t="s">
+      <c r="B7" s="1" t="s">
         <v>52</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="0" t="s">
+      <c r="A8" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="B8" s="0" t="s">
+      <c r="B8" s="1" t="s">
         <v>52</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="0" t="s">
+      <c r="A9" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="B9" s="0" t="s">
+      <c r="B9" s="1" t="s">
         <v>52</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="0" t="s">
+      <c r="A10" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="B10" s="0" t="s">
+      <c r="B10" s="1" t="s">
         <v>53</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="0" t="s">
+      <c r="A11" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="B11" s="0" t="s">
+      <c r="B11" s="1" t="s">
         <v>53</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="0" t="s">
+      <c r="A12" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="B12" s="0" t="s">
+      <c r="B12" s="1" t="s">
         <v>53</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="0" t="s">
+      <c r="A13" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="B13" s="0" t="s">
+      <c r="B13" s="1" t="s">
         <v>53</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="0" t="s">
+      <c r="A14" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="B14" s="0" t="s">
+      <c r="B14" s="1" t="s">
         <v>53</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="0" t="s">
+      <c r="A15" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="B15" s="0" t="s">
+      <c r="B15" s="1" t="s">
         <v>54</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="0" t="s">
+      <c r="A16" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="B16" s="0" t="s">
+      <c r="B16" s="1" t="s">
         <v>54</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="0" t="s">
+      <c r="A17" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="B17" s="0" t="s">
+      <c r="B17" s="1" t="s">
         <v>54</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="0" t="s">
+      <c r="A18" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="B18" s="0" t="s">
+      <c r="B18" s="1" t="s">
         <v>54</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="0" t="s">
+      <c r="A19" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="B19" s="0" t="s">
+      <c r="B19" s="1" t="s">
         <v>54</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="0" t="s">
+      <c r="A20" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="B20" s="0" t="s">
+      <c r="B20" s="1" t="s">
         <v>54</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="0" t="s">
+      <c r="A21" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="B21" s="0" t="s">
+      <c r="B21" s="1" t="s">
         <v>54</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="0" t="s">
+      <c r="A22" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="B22" s="0" t="s">
+      <c r="B22" s="1" t="s">
         <v>54</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="0" t="s">
+      <c r="A23" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="B23" s="0" t="s">
+      <c r="B23" s="1" t="s">
         <v>54</v>
       </c>
     </row>
@@ -1470,566 +1678,776 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:C69"/>
+  <dimension ref="A1:D69"/>
   <sheetFormatPr defaultColWidth="8.83203125" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="42.5"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="40.16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="42.5"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="40.16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="27.08"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="15.24"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16384" min="16382" style="0" width="11.53"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="0" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="0" t="s">
+      <c r="B1" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="C1" s="0" t="s">
+      <c r="C1" s="1" t="s">
         <v>56</v>
       </c>
+      <c r="D1" s="0" t="s">
+        <v>57</v>
+      </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="0" t="s">
+      <c r="A2" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="0" t="s">
-        <v>57</v>
+      <c r="C2" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="D2" s="0" t="s">
+        <v>59</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="0" t="s">
+      <c r="A3" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="C3" s="0" t="s">
-        <v>58</v>
+      <c r="C3" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="D3" s="0" t="s">
+        <v>61</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="0" t="s">
+      <c r="A4" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="C4" s="0" t="s">
-        <v>59</v>
+      <c r="C4" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="D4" s="0" t="s">
+        <v>63</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="0" t="s">
+      <c r="A5" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="C5" s="0" t="s">
-        <v>60</v>
+      <c r="C5" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="D5" s="0" t="s">
+        <v>65</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="0" t="s">
+      <c r="A6" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="C6" s="0" t="s">
-        <v>61</v>
+      <c r="C6" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="D6" s="0" t="s">
+        <v>67</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="0" t="s">
+      <c r="A7" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="C7" s="0" t="s">
-        <v>62</v>
+      <c r="C7" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="D7" s="0" t="s">
+        <v>69</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="0" t="s">
+      <c r="A8" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="C8" s="0" t="s">
-        <v>63</v>
+      <c r="C8" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="D8" s="0" t="s">
+        <v>71</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="0" t="s">
+      <c r="A9" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="C9" s="0" t="s">
-        <v>64</v>
+      <c r="C9" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="D9" s="0" t="s">
+        <v>73</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="0" t="s">
+      <c r="A10" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="C10" s="0" t="s">
-        <v>65</v>
+      <c r="C10" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="D10" s="0" t="s">
+        <v>75</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="0" t="s">
+      <c r="A11" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="C11" s="0" t="s">
-        <v>66</v>
+      <c r="C11" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="D11" s="0" t="s">
+        <v>77</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="0" t="s">
+      <c r="A12" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="C12" s="0" t="s">
-        <v>67</v>
+      <c r="C12" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="D12" s="0" t="s">
+        <v>79</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="0" t="s">
+      <c r="A13" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="C13" s="0" t="s">
-        <v>68</v>
+      <c r="C13" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="D13" s="0" t="s">
+        <v>81</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="0" t="s">
+      <c r="A14" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="C14" s="0" t="s">
-        <v>69</v>
+      <c r="C14" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="D14" s="0" t="s">
+        <v>83</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="0" t="s">
+      <c r="A15" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="C15" s="0" t="s">
-        <v>70</v>
+      <c r="C15" s="1" t="s">
+        <v>84</v>
+      </c>
+      <c r="D15" s="0" t="s">
+        <v>85</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="0" t="s">
+      <c r="A16" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="C16" s="0" t="s">
-        <v>71</v>
+      <c r="C16" s="1" t="s">
+        <v>86</v>
+      </c>
+      <c r="D16" s="0" t="s">
+        <v>87</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="0" t="s">
+      <c r="A17" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="C17" s="0" t="s">
-        <v>72</v>
+      <c r="C17" s="1" t="s">
+        <v>88</v>
+      </c>
+      <c r="D17" s="0" t="s">
+        <v>89</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="0" t="s">
+      <c r="A18" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="C18" s="0" t="s">
-        <v>73</v>
+      <c r="C18" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="D18" s="0" t="s">
+        <v>91</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="0" t="s">
+      <c r="A19" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="C19" s="0" t="s">
-        <v>74</v>
+      <c r="C19" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="D19" s="0" t="s">
+        <v>93</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="0" t="s">
+      <c r="A20" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="C20" s="0" t="s">
-        <v>75</v>
+      <c r="C20" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="D20" s="0" t="s">
+        <v>95</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="0" t="s">
+      <c r="A21" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="C21" s="0" t="s">
-        <v>76</v>
+      <c r="C21" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="D21" s="0" t="s">
+        <v>97</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="0" t="s">
+      <c r="A22" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="C22" s="0" t="s">
-        <v>77</v>
+      <c r="C22" s="1" t="s">
+        <v>98</v>
+      </c>
+      <c r="D22" s="0" t="s">
+        <v>99</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="0" t="s">
+      <c r="A23" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="C23" s="0" t="s">
-        <v>78</v>
+      <c r="C23" s="1" t="s">
+        <v>100</v>
+      </c>
+      <c r="D23" s="0" t="s">
+        <v>101</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="0" t="s">
+      <c r="A24" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="C24" s="0" t="s">
-        <v>79</v>
+      <c r="C24" s="1" t="s">
+        <v>102</v>
+      </c>
+      <c r="D24" s="0" t="s">
+        <v>103</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="0" t="s">
+      <c r="A25" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="C25" s="0" t="s">
-        <v>80</v>
+      <c r="C25" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="D25" s="0" t="s">
+        <v>105</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="0" t="s">
+      <c r="A26" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="C26" s="0" t="s">
-        <v>81</v>
+      <c r="C26" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="D26" s="0" t="s">
+        <v>107</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="0" t="s">
+      <c r="A27" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="C27" s="0" t="s">
-        <v>82</v>
+      <c r="C27" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="D27" s="0" t="s">
+        <v>109</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="0" t="s">
+      <c r="A28" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="C28" s="0" t="s">
-        <v>83</v>
+      <c r="C28" s="1" t="s">
+        <v>110</v>
+      </c>
+      <c r="D28" s="0" t="s">
+        <v>111</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="0" t="s">
+      <c r="A29" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="C29" s="0" t="s">
-        <v>84</v>
+      <c r="C29" s="1" t="s">
+        <v>112</v>
+      </c>
+      <c r="D29" s="0" t="s">
+        <v>113</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="0" t="s">
+      <c r="A30" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="C30" s="0" t="s">
-        <v>85</v>
+      <c r="C30" s="1" t="s">
+        <v>114</v>
+      </c>
+      <c r="D30" s="0" t="s">
+        <v>115</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="0" t="s">
+      <c r="A31" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="C31" s="0" t="s">
-        <v>86</v>
+      <c r="C31" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="D31" s="0" t="s">
+        <v>117</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="0" t="s">
+      <c r="A32" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="C32" s="0" t="s">
-        <v>87</v>
+      <c r="C32" s="1" t="s">
+        <v>118</v>
+      </c>
+      <c r="D32" s="0" t="s">
+        <v>119</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="0" t="s">
+      <c r="A33" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="C33" s="0" t="s">
-        <v>88</v>
+      <c r="C33" s="1" t="s">
+        <v>120</v>
+      </c>
+      <c r="D33" s="0" t="s">
+        <v>121</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="0" t="s">
+      <c r="A34" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="C34" s="0" t="s">
-        <v>89</v>
+      <c r="C34" s="1" t="s">
+        <v>122</v>
+      </c>
+      <c r="D34" s="0" t="s">
+        <v>123</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="0" t="s">
+      <c r="A35" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="C35" s="0" t="s">
-        <v>90</v>
+      <c r="C35" s="1" t="s">
+        <v>124</v>
+      </c>
+      <c r="D35" s="0" t="s">
+        <v>125</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A36" s="0" t="s">
+      <c r="A36" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="C36" s="0" t="s">
-        <v>91</v>
+      <c r="C36" s="1" t="s">
+        <v>126</v>
+      </c>
+      <c r="D36" s="0" t="s">
+        <v>127</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A37" s="0" t="s">
+      <c r="A37" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="C37" s="0" t="s">
-        <v>92</v>
+      <c r="C37" s="1" t="s">
+        <v>128</v>
+      </c>
+      <c r="D37" s="0" t="s">
+        <v>129</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A38" s="0" t="s">
+      <c r="A38" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="C38" s="0" t="s">
-        <v>93</v>
+      <c r="C38" s="1" t="s">
+        <v>130</v>
+      </c>
+      <c r="D38" s="0" t="s">
+        <v>131</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A39" s="0" t="s">
+      <c r="A39" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="C39" s="0" t="s">
-        <v>94</v>
+      <c r="C39" s="1" t="s">
+        <v>132</v>
+      </c>
+      <c r="D39" s="0" t="s">
+        <v>133</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A40" s="0" t="s">
+      <c r="A40" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="C40" s="0" t="s">
-        <v>95</v>
+      <c r="C40" s="1" t="s">
+        <v>134</v>
+      </c>
+      <c r="D40" s="0" t="s">
+        <v>135</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A41" s="0" t="s">
+      <c r="A41" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="C41" s="0" t="s">
-        <v>96</v>
+      <c r="C41" s="1" t="s">
+        <v>136</v>
+      </c>
+      <c r="D41" s="0" t="s">
+        <v>137</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A42" s="0" t="s">
+      <c r="A42" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="C42" s="0" t="s">
-        <v>97</v>
+      <c r="C42" s="1" t="s">
+        <v>138</v>
+      </c>
+      <c r="D42" s="0" t="s">
+        <v>139</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A43" s="0" t="s">
+      <c r="A43" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="C43" s="0" t="s">
-        <v>98</v>
+      <c r="C43" s="1" t="s">
+        <v>140</v>
+      </c>
+      <c r="D43" s="0" t="s">
+        <v>141</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A44" s="0" t="s">
+      <c r="A44" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="C44" s="0" t="s">
-        <v>99</v>
+      <c r="C44" s="1" t="s">
+        <v>142</v>
+      </c>
+      <c r="D44" s="0" t="s">
+        <v>143</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A45" s="0" t="s">
+      <c r="A45" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="C45" s="0" t="s">
-        <v>100</v>
+      <c r="C45" s="1" t="s">
+        <v>144</v>
+      </c>
+      <c r="D45" s="0" t="s">
+        <v>145</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A46" s="0" t="s">
+      <c r="A46" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="C46" s="0" t="s">
-        <v>101</v>
+      <c r="C46" s="1" t="s">
+        <v>146</v>
+      </c>
+      <c r="D46" s="0" t="s">
+        <v>147</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A47" s="0" t="s">
+      <c r="A47" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="C47" s="0" t="s">
-        <v>102</v>
+      <c r="C47" s="1" t="s">
+        <v>148</v>
+      </c>
+      <c r="D47" s="0" t="s">
+        <v>149</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A48" s="0" t="s">
+      <c r="A48" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="C48" s="0" t="s">
-        <v>103</v>
+      <c r="C48" s="1" t="s">
+        <v>150</v>
+      </c>
+      <c r="D48" s="0" t="s">
+        <v>151</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A49" s="0" t="s">
+      <c r="A49" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="C49" s="0" t="s">
-        <v>104</v>
+      <c r="C49" s="1" t="s">
+        <v>152</v>
+      </c>
+      <c r="D49" s="0" t="s">
+        <v>153</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A50" s="0" t="s">
+      <c r="A50" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="C50" s="0" t="s">
-        <v>105</v>
+      <c r="C50" s="1" t="s">
+        <v>154</v>
+      </c>
+      <c r="D50" s="0" t="s">
+        <v>155</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A51" s="0" t="s">
+      <c r="A51" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="C51" s="0" t="s">
-        <v>106</v>
+      <c r="C51" s="1" t="s">
+        <v>156</v>
+      </c>
+      <c r="D51" s="0" t="s">
+        <v>157</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A52" s="0" t="s">
+      <c r="A52" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="C52" s="0" t="s">
-        <v>107</v>
+      <c r="C52" s="1" t="s">
+        <v>158</v>
+      </c>
+      <c r="D52" s="0" t="s">
+        <v>159</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A53" s="0" t="s">
+      <c r="A53" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="C53" s="0" t="s">
-        <v>108</v>
+      <c r="C53" s="1" t="s">
+        <v>160</v>
+      </c>
+      <c r="D53" s="0" t="s">
+        <v>161</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A54" s="0" t="s">
+      <c r="A54" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="C54" s="0" t="s">
-        <v>109</v>
+      <c r="C54" s="1" t="s">
+        <v>162</v>
+      </c>
+      <c r="D54" s="0" t="s">
+        <v>163</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A55" s="0" t="s">
+      <c r="A55" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="C55" s="0" t="s">
-        <v>110</v>
+      <c r="C55" s="1" t="s">
+        <v>164</v>
+      </c>
+      <c r="D55" s="0" t="s">
+        <v>165</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A56" s="0" t="s">
+      <c r="A56" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="C56" s="0" t="s">
-        <v>111</v>
+      <c r="C56" s="1" t="s">
+        <v>166</v>
+      </c>
+      <c r="D56" s="0" t="s">
+        <v>167</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A57" s="0" t="s">
+      <c r="A57" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="C57" s="0" t="s">
-        <v>112</v>
+      <c r="C57" s="1" t="s">
+        <v>168</v>
+      </c>
+      <c r="D57" s="0" t="s">
+        <v>169</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A58" s="0" t="s">
+      <c r="A58" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="C58" s="0" t="s">
-        <v>113</v>
+      <c r="C58" s="1" t="s">
+        <v>170</v>
+      </c>
+      <c r="D58" s="0" t="s">
+        <v>171</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A59" s="0" t="s">
+      <c r="A59" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="C59" s="0" t="s">
-        <v>114</v>
+      <c r="C59" s="1" t="s">
+        <v>172</v>
+      </c>
+      <c r="D59" s="0" t="s">
+        <v>173</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A60" s="0" t="s">
+      <c r="A60" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="C60" s="0" t="s">
-        <v>115</v>
+      <c r="C60" s="1" t="s">
+        <v>174</v>
+      </c>
+      <c r="D60" s="0" t="s">
+        <v>175</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A61" s="0" t="s">
+      <c r="A61" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="C61" s="0" t="s">
-        <v>116</v>
+      <c r="C61" s="1" t="s">
+        <v>176</v>
+      </c>
+      <c r="D61" s="0" t="s">
+        <v>177</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A62" s="0" t="s">
+      <c r="A62" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="C62" s="0" t="s">
-        <v>117</v>
+      <c r="C62" s="1" t="s">
+        <v>178</v>
+      </c>
+      <c r="D62" s="0" t="s">
+        <v>179</v>
       </c>
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A63" s="0" t="s">
+      <c r="A63" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="C63" s="0" t="s">
-        <v>118</v>
+      <c r="C63" s="1" t="s">
+        <v>180</v>
+      </c>
+      <c r="D63" s="0" t="s">
+        <v>181</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A64" s="0" t="s">
+      <c r="A64" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="C64" s="0" t="s">
-        <v>119</v>
+      <c r="C64" s="1" t="s">
+        <v>182</v>
+      </c>
+      <c r="D64" s="0" t="s">
+        <v>183</v>
       </c>
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A65" s="0" t="s">
+      <c r="A65" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="C65" s="0" t="s">
-        <v>120</v>
+      <c r="C65" s="1" t="s">
+        <v>184</v>
+      </c>
+      <c r="D65" s="0" t="s">
+        <v>185</v>
       </c>
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A66" s="0" t="s">
+      <c r="A66" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="C66" s="0" t="s">
-        <v>121</v>
+      <c r="C66" s="1" t="s">
+        <v>186</v>
+      </c>
+      <c r="D66" s="0" t="s">
+        <v>187</v>
       </c>
     </row>
     <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A67" s="0" t="s">
+      <c r="A67" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="C67" s="0" t="s">
-        <v>122</v>
+      <c r="C67" s="1" t="s">
+        <v>188</v>
+      </c>
+      <c r="D67" s="0" t="s">
+        <v>189</v>
       </c>
     </row>
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A68" s="0" t="s">
+      <c r="A68" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="C68" s="0" t="s">
-        <v>123</v>
+      <c r="C68" s="1" t="s">
+        <v>190</v>
+      </c>
+      <c r="D68" s="0" t="s">
+        <v>191</v>
       </c>
     </row>
     <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A69" s="0" t="s">
+      <c r="A69" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="C69" s="0" t="s">
-        <v>124</v>
+      <c r="C69" s="1" t="s">
+        <v>192</v>
+      </c>
+      <c r="D69" s="0" t="s">
+        <v>193</v>
       </c>
     </row>
   </sheetData>
@@ -2051,590 +2469,590 @@
   <dimension ref="A1:F29"/>
   <sheetFormatPr defaultColWidth="8.83203125" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="1" style="0" width="51"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="3" style="0" width="33.51"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="27.83"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="53.83"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="1" style="1" width="51"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="3" style="1" width="33.52"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="27.83"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="53.83"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="0" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="0" t="s">
+      <c r="B1" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="C1" s="0" t="s">
-        <v>125</v>
-      </c>
-      <c r="D1" s="0" t="s">
-        <v>126</v>
-      </c>
-      <c r="E1" s="0" t="s">
-        <v>127</v>
-      </c>
-      <c r="F1" s="0" t="s">
-        <v>128</v>
+      <c r="C1" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>194</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>195</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>196</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="0" t="s">
+      <c r="A2" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B2" s="0" t="s">
-        <v>62</v>
-      </c>
-      <c r="C2" s="0" t="s">
-        <v>129</v>
-      </c>
-      <c r="D2" s="0" t="s">
-        <v>130</v>
-      </c>
-      <c r="E2" s="0" t="s">
-        <v>131</v>
-      </c>
-      <c r="F2" s="0" t="s">
-        <v>132</v>
+      <c r="B2" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>197</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>198</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>199</v>
+      </c>
+      <c r="F2" s="1" t="s">
+        <v>200</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="0" t="s">
+      <c r="A3" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="B3" s="0" t="s">
-        <v>67</v>
-      </c>
-      <c r="C3" s="0" t="s">
-        <v>133</v>
-      </c>
-      <c r="D3" s="0" t="s">
-        <v>130</v>
-      </c>
-      <c r="E3" s="0" t="s">
-        <v>131</v>
-      </c>
-      <c r="F3" s="0" t="s">
-        <v>134</v>
+      <c r="B3" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>201</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>198</v>
+      </c>
+      <c r="E3" s="1" t="s">
+        <v>199</v>
+      </c>
+      <c r="F3" s="1" t="s">
+        <v>202</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="0" t="s">
+      <c r="A4" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="B4" s="0" t="s">
-        <v>71</v>
-      </c>
-      <c r="C4" s="0" t="s">
-        <v>135</v>
-      </c>
-      <c r="D4" s="0" t="s">
-        <v>130</v>
-      </c>
-      <c r="E4" s="0" t="s">
-        <v>131</v>
-      </c>
-      <c r="F4" s="0" t="s">
-        <v>136</v>
+      <c r="B4" s="1" t="s">
+        <v>86</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>203</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>198</v>
+      </c>
+      <c r="E4" s="1" t="s">
+        <v>199</v>
+      </c>
+      <c r="F4" s="1" t="s">
+        <v>204</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="0" t="s">
+      <c r="A5" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="B5" s="0" t="s">
-        <v>72</v>
-      </c>
-      <c r="C5" s="0" t="s">
-        <v>137</v>
-      </c>
-      <c r="D5" s="0" t="s">
-        <v>130</v>
-      </c>
-      <c r="E5" s="0" t="s">
-        <v>131</v>
-      </c>
-      <c r="F5" s="0" t="s">
+      <c r="B5" s="1" t="s">
+        <v>88</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>205</v>
+      </c>
+      <c r="D5" s="1" t="s">
+        <v>198</v>
+      </c>
+      <c r="E5" s="1" t="s">
+        <v>199</v>
+      </c>
+      <c r="F5" s="1" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>98</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>207</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>198</v>
+      </c>
+      <c r="E6" s="1" t="s">
+        <v>199</v>
+      </c>
+      <c r="F6" s="1" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>209</v>
+      </c>
+      <c r="D7" s="1" t="s">
+        <v>198</v>
+      </c>
+      <c r="E7" s="1" t="s">
+        <v>199</v>
+      </c>
+      <c r="F7" s="1" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="B8" s="1" t="s">
+        <v>110</v>
+      </c>
+      <c r="C8" s="1" t="s">
+        <v>211</v>
+      </c>
+      <c r="D8" s="1" t="s">
+        <v>198</v>
+      </c>
+      <c r="E8" s="1" t="s">
+        <v>199</v>
+      </c>
+      <c r="F8" s="1" t="s">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="B9" s="1" t="s">
+        <v>122</v>
+      </c>
+      <c r="C9" s="1" t="s">
+        <v>213</v>
+      </c>
+      <c r="D9" s="1" t="s">
+        <v>198</v>
+      </c>
+      <c r="E9" s="1" t="s">
+        <v>199</v>
+      </c>
+      <c r="F9" s="1" t="s">
+        <v>214</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="B10" s="1" t="s">
         <v>138</v>
       </c>
-    </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="0" t="s">
-        <v>12</v>
-      </c>
-      <c r="B6" s="0" t="s">
-        <v>77</v>
-      </c>
-      <c r="C6" s="0" t="s">
-        <v>139</v>
-      </c>
-      <c r="D6" s="0" t="s">
-        <v>130</v>
-      </c>
-      <c r="E6" s="0" t="s">
-        <v>131</v>
-      </c>
-      <c r="F6" s="0" t="s">
-        <v>140</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="0" t="s">
-        <v>14</v>
-      </c>
-      <c r="B7" s="0" t="s">
-        <v>80</v>
-      </c>
-      <c r="C7" s="0" t="s">
-        <v>141</v>
-      </c>
-      <c r="D7" s="0" t="s">
-        <v>130</v>
-      </c>
-      <c r="E7" s="0" t="s">
-        <v>131</v>
-      </c>
-      <c r="F7" s="0" t="s">
-        <v>142</v>
-      </c>
-    </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="0" t="s">
-        <v>16</v>
-      </c>
-      <c r="B8" s="0" t="s">
-        <v>83</v>
-      </c>
-      <c r="C8" s="0" t="s">
-        <v>143</v>
-      </c>
-      <c r="D8" s="0" t="s">
-        <v>130</v>
-      </c>
-      <c r="E8" s="0" t="s">
-        <v>131</v>
-      </c>
-      <c r="F8" s="0" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="0" t="s">
-        <v>18</v>
-      </c>
-      <c r="B9" s="0" t="s">
-        <v>89</v>
-      </c>
-      <c r="C9" s="0" t="s">
-        <v>145</v>
-      </c>
-      <c r="D9" s="0" t="s">
-        <v>130</v>
-      </c>
-      <c r="E9" s="0" t="s">
-        <v>131</v>
-      </c>
-      <c r="F9" s="0" t="s">
+      <c r="C10" s="1" t="s">
+        <v>215</v>
+      </c>
+      <c r="D10" s="1" t="s">
+        <v>216</v>
+      </c>
+      <c r="E10" s="1" t="s">
+        <v>199</v>
+      </c>
+      <c r="F10" s="1" t="s">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="B11" s="1" t="s">
+        <v>138</v>
+      </c>
+      <c r="C11" s="1" t="s">
+        <v>218</v>
+      </c>
+      <c r="D11" s="1" t="s">
+        <v>198</v>
+      </c>
+      <c r="E11" s="1" t="s">
+        <v>199</v>
+      </c>
+      <c r="F11" s="1" t="s">
+        <v>219</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="B12" s="1" t="s">
         <v>146</v>
       </c>
-    </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="0" t="s">
-        <v>30</v>
-      </c>
-      <c r="B10" s="0" t="s">
-        <v>97</v>
-      </c>
-      <c r="C10" s="0" t="s">
-        <v>147</v>
-      </c>
-      <c r="D10" s="0" t="s">
+      <c r="C12" s="1" t="s">
+        <v>220</v>
+      </c>
+      <c r="D12" s="1" t="s">
+        <v>216</v>
+      </c>
+      <c r="E12" s="1" t="s">
+        <v>199</v>
+      </c>
+      <c r="F12" s="1" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="B13" s="1" t="s">
+        <v>146</v>
+      </c>
+      <c r="C13" s="1" t="s">
+        <v>222</v>
+      </c>
+      <c r="D13" s="1" t="s">
+        <v>198</v>
+      </c>
+      <c r="E13" s="1" t="s">
+        <v>199</v>
+      </c>
+      <c r="F13" s="1" t="s">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="B14" s="1" t="s">
         <v>148</v>
       </c>
-      <c r="E10" s="0" t="s">
-        <v>131</v>
-      </c>
-      <c r="F10" s="0" t="s">
-        <v>149</v>
-      </c>
-    </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="0" t="s">
-        <v>30</v>
-      </c>
-      <c r="B11" s="0" t="s">
-        <v>97</v>
-      </c>
-      <c r="C11" s="0" t="s">
-        <v>150</v>
-      </c>
-      <c r="D11" s="0" t="s">
-        <v>130</v>
-      </c>
-      <c r="E11" s="0" t="s">
-        <v>131</v>
-      </c>
-      <c r="F11" s="0" t="s">
-        <v>151</v>
-      </c>
-    </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="1" t="s">
+      <c r="C14" s="1" t="s">
+        <v>224</v>
+      </c>
+      <c r="D14" s="1" t="s">
+        <v>198</v>
+      </c>
+      <c r="E14" s="1" t="s">
+        <v>199</v>
+      </c>
+      <c r="F14" s="1" t="s">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="B12" s="0" t="s">
-        <v>101</v>
-      </c>
-      <c r="C12" s="0" t="s">
+      <c r="B15" s="1" t="s">
+        <v>148</v>
+      </c>
+      <c r="C15" s="1" t="s">
+        <v>225</v>
+      </c>
+      <c r="D15" s="1" t="s">
+        <v>216</v>
+      </c>
+      <c r="E15" s="1" t="s">
+        <v>199</v>
+      </c>
+      <c r="F15" s="1" t="s">
+        <v>226</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="B16" s="1" t="s">
         <v>152</v>
       </c>
-      <c r="D12" s="0" t="s">
-        <v>148</v>
-      </c>
-      <c r="E12" s="0" t="s">
-        <v>131</v>
-      </c>
-      <c r="F12" s="0" t="s">
-        <v>153</v>
-      </c>
-    </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="0" t="s">
-        <v>32</v>
-      </c>
-      <c r="B13" s="0" t="s">
-        <v>101</v>
-      </c>
-      <c r="C13" s="0" t="s">
-        <v>154</v>
-      </c>
-      <c r="D13" s="0" t="s">
-        <v>130</v>
-      </c>
-      <c r="E13" s="0" t="s">
-        <v>131</v>
-      </c>
-      <c r="F13" s="0" t="s">
-        <v>155</v>
-      </c>
-    </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="0" t="s">
-        <v>32</v>
-      </c>
-      <c r="B14" s="0" t="s">
-        <v>102</v>
-      </c>
-      <c r="C14" s="0" t="s">
-        <v>156</v>
-      </c>
-      <c r="D14" s="0" t="s">
-        <v>130</v>
-      </c>
-      <c r="E14" s="0" t="s">
-        <v>131</v>
-      </c>
-      <c r="F14" s="0" t="s">
-        <v>155</v>
-      </c>
-    </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="0" t="s">
-        <v>32</v>
-      </c>
-      <c r="B15" s="0" t="s">
-        <v>102</v>
-      </c>
-      <c r="C15" s="0" t="s">
-        <v>157</v>
-      </c>
-      <c r="D15" s="0" t="s">
-        <v>148</v>
-      </c>
-      <c r="E15" s="0" t="s">
-        <v>131</v>
-      </c>
-      <c r="F15" s="0" t="s">
-        <v>158</v>
-      </c>
-    </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="0" t="s">
+      <c r="C16" s="1" t="s">
+        <v>227</v>
+      </c>
+      <c r="D16" s="1" t="s">
+        <v>216</v>
+      </c>
+      <c r="E16" s="1" t="s">
+        <v>199</v>
+      </c>
+      <c r="F16" s="1" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="B16" s="0" t="s">
-        <v>104</v>
-      </c>
-      <c r="C16" s="0" t="s">
-        <v>159</v>
-      </c>
-      <c r="D16" s="0" t="s">
-        <v>148</v>
-      </c>
-      <c r="E16" s="0" t="s">
-        <v>131</v>
-      </c>
-      <c r="F16" s="0" t="s">
+      <c r="B17" s="1" t="s">
+        <v>152</v>
+      </c>
+      <c r="C17" s="1" t="s">
+        <v>229</v>
+      </c>
+      <c r="D17" s="1" t="s">
+        <v>198</v>
+      </c>
+      <c r="E17" s="1" t="s">
+        <v>199</v>
+      </c>
+      <c r="F17" s="1" t="s">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="B18" s="1" t="s">
         <v>160</v>
       </c>
-    </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="0" t="s">
-        <v>34</v>
-      </c>
-      <c r="B17" s="0" t="s">
-        <v>104</v>
-      </c>
-      <c r="C17" s="0" t="s">
-        <v>161</v>
-      </c>
-      <c r="D17" s="0" t="s">
-        <v>130</v>
-      </c>
-      <c r="E17" s="0" t="s">
-        <v>131</v>
-      </c>
-      <c r="F17" s="0" t="s">
-        <v>162</v>
-      </c>
-    </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="0" t="s">
+      <c r="C18" s="1" t="s">
+        <v>231</v>
+      </c>
+      <c r="D18" s="1" t="s">
+        <v>198</v>
+      </c>
+      <c r="E18" s="1" t="s">
+        <v>199</v>
+      </c>
+      <c r="F18" s="1" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="B18" s="0" t="s">
-        <v>108</v>
-      </c>
-      <c r="C18" s="0" t="s">
-        <v>163</v>
-      </c>
-      <c r="D18" s="0" t="s">
-        <v>130</v>
-      </c>
-      <c r="E18" s="0" t="s">
-        <v>131</v>
-      </c>
-      <c r="F18" s="0" t="s">
-        <v>164</v>
-      </c>
-    </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="0" t="s">
-        <v>36</v>
-      </c>
-      <c r="B19" s="0" t="s">
-        <v>108</v>
-      </c>
-      <c r="C19" s="0" t="s">
-        <v>165</v>
-      </c>
-      <c r="D19" s="0" t="s">
-        <v>148</v>
-      </c>
-      <c r="E19" s="0" t="s">
-        <v>131</v>
-      </c>
-      <c r="F19" s="0" t="s">
+      <c r="B19" s="1" t="s">
+        <v>160</v>
+      </c>
+      <c r="C19" s="1" t="s">
+        <v>233</v>
+      </c>
+      <c r="D19" s="1" t="s">
+        <v>216</v>
+      </c>
+      <c r="E19" s="1" t="s">
+        <v>199</v>
+      </c>
+      <c r="F19" s="1" t="s">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="B20" s="1" t="s">
         <v>166</v>
       </c>
-    </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="0" t="s">
+      <c r="C20" s="1" t="s">
+        <v>235</v>
+      </c>
+      <c r="D20" s="1" t="s">
+        <v>216</v>
+      </c>
+      <c r="E20" s="1" t="s">
+        <v>199</v>
+      </c>
+      <c r="F20" s="1" t="s">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="B20" s="0" t="s">
-        <v>111</v>
-      </c>
-      <c r="C20" s="0" t="s">
-        <v>167</v>
-      </c>
-      <c r="D20" s="0" t="s">
-        <v>148</v>
-      </c>
-      <c r="E20" s="0" t="s">
-        <v>131</v>
-      </c>
-      <c r="F20" s="0" t="s">
-        <v>168</v>
-      </c>
-    </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="0" t="s">
-        <v>38</v>
-      </c>
-      <c r="B21" s="0" t="s">
-        <v>111</v>
-      </c>
-      <c r="C21" s="0" t="s">
-        <v>169</v>
-      </c>
-      <c r="D21" s="0" t="s">
-        <v>130</v>
-      </c>
-      <c r="E21" s="0" t="s">
-        <v>131</v>
-      </c>
-      <c r="F21" s="0" t="s">
-        <v>170</v>
+      <c r="B21" s="1" t="s">
+        <v>166</v>
+      </c>
+      <c r="C21" s="1" t="s">
+        <v>237</v>
+      </c>
+      <c r="D21" s="1" t="s">
+        <v>198</v>
+      </c>
+      <c r="E21" s="1" t="s">
+        <v>199</v>
+      </c>
+      <c r="F21" s="1" t="s">
+        <v>238</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="0" t="s">
+      <c r="A22" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="B22" s="0" t="s">
-        <v>115</v>
-      </c>
-      <c r="C22" s="0" t="s">
-        <v>171</v>
-      </c>
-      <c r="D22" s="0" t="s">
-        <v>130</v>
-      </c>
-      <c r="E22" s="0" t="s">
-        <v>131</v>
-      </c>
-      <c r="F22" s="0" t="s">
-        <v>162</v>
+      <c r="B22" s="1" t="s">
+        <v>174</v>
+      </c>
+      <c r="C22" s="1" t="s">
+        <v>239</v>
+      </c>
+      <c r="D22" s="1" t="s">
+        <v>198</v>
+      </c>
+      <c r="E22" s="1" t="s">
+        <v>199</v>
+      </c>
+      <c r="F22" s="1" t="s">
+        <v>230</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="0" t="s">
+      <c r="A23" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="B23" s="0" t="s">
-        <v>115</v>
-      </c>
-      <c r="C23" s="0" t="s">
-        <v>172</v>
-      </c>
-      <c r="D23" s="0" t="s">
-        <v>148</v>
-      </c>
-      <c r="E23" s="0" t="s">
-        <v>131</v>
-      </c>
-      <c r="F23" s="0" t="s">
-        <v>160</v>
+      <c r="B23" s="1" t="s">
+        <v>174</v>
+      </c>
+      <c r="C23" s="1" t="s">
+        <v>240</v>
+      </c>
+      <c r="D23" s="1" t="s">
+        <v>216</v>
+      </c>
+      <c r="E23" s="1" t="s">
+        <v>199</v>
+      </c>
+      <c r="F23" s="1" t="s">
+        <v>228</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="0" t="s">
+      <c r="A24" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="B24" s="0" t="s">
-        <v>117</v>
-      </c>
-      <c r="C24" s="0" t="s">
-        <v>173</v>
-      </c>
-      <c r="D24" s="0" t="s">
-        <v>130</v>
-      </c>
-      <c r="E24" s="0" t="s">
-        <v>131</v>
-      </c>
-      <c r="F24" s="0" t="s">
-        <v>162</v>
+      <c r="B24" s="1" t="s">
+        <v>178</v>
+      </c>
+      <c r="C24" s="1" t="s">
+        <v>241</v>
+      </c>
+      <c r="D24" s="1" t="s">
+        <v>198</v>
+      </c>
+      <c r="E24" s="1" t="s">
+        <v>199</v>
+      </c>
+      <c r="F24" s="1" t="s">
+        <v>230</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="0" t="s">
+      <c r="A25" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="B25" s="0" t="s">
-        <v>117</v>
-      </c>
-      <c r="C25" s="0" t="s">
-        <v>174</v>
-      </c>
-      <c r="D25" s="0" t="s">
-        <v>148</v>
-      </c>
-      <c r="E25" s="0" t="s">
-        <v>131</v>
-      </c>
-      <c r="F25" s="0" t="s">
-        <v>160</v>
+      <c r="B25" s="1" t="s">
+        <v>178</v>
+      </c>
+      <c r="C25" s="1" t="s">
+        <v>242</v>
+      </c>
+      <c r="D25" s="1" t="s">
+        <v>216</v>
+      </c>
+      <c r="E25" s="1" t="s">
+        <v>199</v>
+      </c>
+      <c r="F25" s="1" t="s">
+        <v>228</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="1" t="s">
+      <c r="A26" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="B26" s="0" t="s">
-        <v>119</v>
-      </c>
-      <c r="C26" s="0" t="s">
-        <v>175</v>
-      </c>
-      <c r="D26" s="0" t="s">
-        <v>130</v>
-      </c>
-      <c r="E26" s="0" t="s">
-        <v>131</v>
-      </c>
-      <c r="F26" s="0" t="s">
-        <v>162</v>
+      <c r="B26" s="1" t="s">
+        <v>182</v>
+      </c>
+      <c r="C26" s="1" t="s">
+        <v>243</v>
+      </c>
+      <c r="D26" s="1" t="s">
+        <v>198</v>
+      </c>
+      <c r="E26" s="1" t="s">
+        <v>199</v>
+      </c>
+      <c r="F26" s="1" t="s">
+        <v>230</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="0" t="s">
+      <c r="A27" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="B27" s="0" t="s">
-        <v>119</v>
-      </c>
-      <c r="C27" s="0" t="s">
-        <v>176</v>
-      </c>
-      <c r="D27" s="0" t="s">
-        <v>148</v>
-      </c>
-      <c r="E27" s="0" t="s">
-        <v>131</v>
-      </c>
-      <c r="F27" s="0" t="s">
-        <v>160</v>
+      <c r="B27" s="1" t="s">
+        <v>182</v>
+      </c>
+      <c r="C27" s="1" t="s">
+        <v>244</v>
+      </c>
+      <c r="D27" s="1" t="s">
+        <v>216</v>
+      </c>
+      <c r="E27" s="1" t="s">
+        <v>199</v>
+      </c>
+      <c r="F27" s="1" t="s">
+        <v>228</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="0" t="s">
+      <c r="A28" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="B28" s="0" t="s">
-        <v>124</v>
-      </c>
-      <c r="C28" s="0" t="s">
-        <v>177</v>
-      </c>
-      <c r="D28" s="0" t="s">
-        <v>130</v>
-      </c>
-      <c r="E28" s="0" t="s">
-        <v>131</v>
-      </c>
-      <c r="F28" s="0" t="s">
-        <v>155</v>
+      <c r="B28" s="1" t="s">
+        <v>192</v>
+      </c>
+      <c r="C28" s="1" t="s">
+        <v>245</v>
+      </c>
+      <c r="D28" s="1" t="s">
+        <v>198</v>
+      </c>
+      <c r="E28" s="1" t="s">
+        <v>199</v>
+      </c>
+      <c r="F28" s="1" t="s">
+        <v>223</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="0" t="s">
+      <c r="A29" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="B29" s="0" t="s">
-        <v>124</v>
-      </c>
-      <c r="C29" s="0" t="s">
-        <v>178</v>
-      </c>
-      <c r="D29" s="0" t="s">
-        <v>148</v>
-      </c>
-      <c r="E29" s="0" t="s">
-        <v>131</v>
-      </c>
-      <c r="F29" s="0" t="s">
-        <v>179</v>
+      <c r="B29" s="1" t="s">
+        <v>192</v>
+      </c>
+      <c r="C29" s="1" t="s">
+        <v>246</v>
+      </c>
+      <c r="D29" s="1" t="s">
+        <v>216</v>
+      </c>
+      <c r="E29" s="1" t="s">
+        <v>199</v>
+      </c>
+      <c r="F29" s="1" t="s">
+        <v>247</v>
       </c>
     </row>
   </sheetData>

</xml_diff>